<commit_message>
Fixes done after End Mar
</commit_message>
<xml_diff>
--- a/Encollect_Web_SCB_P1/Cypress/fixtures/AgencyTemplate.xlsx
+++ b/Encollect_Web_SCB_P1/Cypress/fixtures/AgencyTemplate.xlsx
@@ -401,61 +401,61 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="str">
-        <v>Zita</v>
+        <v>Lilyan</v>
       </c>
       <c r="B2" t="str">
-        <v>O'Kon</v>
+        <v>Jones</v>
       </c>
       <c r="C2" t="str">
-        <v>JSPP9E</v>
+        <v>YSAQZD</v>
       </c>
       <c r="D2" t="str">
-        <v>Jedidiah_Gulgowski1@yahoo.com</v>
+        <v>Kristy_Wolf@hotmail.com</v>
       </c>
       <c r="E2" t="str">
-        <v>kcmaqBk4</v>
+        <v>5YUb5Y1i</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-13</v>
+        <v>2025-09-28</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-02-27</v>
+        <v>2025-08-29</v>
       </c>
       <c r="H2" t="str">
-        <v>0hQVvzwMfw</v>
+        <v>vvsztZmq32</v>
       </c>
       <c r="I2" t="str">
-        <v>Automotive</v>
+        <v>Jewelry</v>
       </c>
       <c r="J2" t="str">
-        <v>Product Accounts Director</v>
+        <v>Dynamic Group Specialist</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-02-28</v>
+        <v>2025-06-02</v>
       </c>
       <c r="L2" t="str">
-        <v>9290704331</v>
+        <v>7051413052</v>
       </c>
       <c r="M2" t="str">
-        <v>Jade70@hotmail.com</v>
+        <v>Cecelia88@yahoo.com</v>
       </c>
       <c r="N2" t="str">
-        <v>Layne</v>
+        <v>Hobart</v>
       </c>
       <c r="O2" t="str">
-        <v>68629 County Line Road</v>
+        <v>5815 Vincent Causeway</v>
       </c>
       <c r="P2" t="str">
-        <v>70658</v>
+        <v>39978</v>
       </c>
       <c r="Q2" t="str">
-        <v>2026-01-20</v>
+        <v>2026-03-15</v>
       </c>
       <c r="R2" t="str">
-        <v>2026-03-08</v>
+        <v>2025-10-05</v>
       </c>
       <c r="S2" t="str">
-        <v>2026-07-06</v>
+        <v>2026-11-05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>